<commit_message>
feat: flag first-gen students and route unmatched campus 76 by earned credits
First-gen is an optional Yes flag before 1st Outreach, not a group tab. Campus 76 still matches control-file lists first, then unmatched students split at 45 earned credits.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/sample_data/contact_report_sample.xlsx
+++ b/sample_data/contact_report_sample.xlsx
@@ -936,11 +936,11 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Boca Raton</t>
+          <t>76</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Jupiter</t>
+          <t>76</t>
         </is>
       </c>
       <c r="G36" t="n">

</xml_diff>